<commit_message>
Fix SIAL workbook hyperlink XML ordering for Excel compatibility
</commit_message>
<xml_diff>
--- a/task-projects/sial-exhibition/attachments/SIAL-Healthy-Companies-MADA.xlsx
+++ b/task-projects/sial-exhibition/attachments/SIAL-Healthy-Companies-MADA.xlsx
@@ -5977,7 +5977,6 @@
       <x:formula>OR(LEFT(G9,3)="غير",LEFT(G9,2)="لم")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:hyperlinks>
     <x:hyperlink r:id="rIdSial9" ref="N9"/>
     <x:hyperlink r:id="rIdSial10" ref="N10"/>
@@ -6090,6 +6089,7 @@
     <x:hyperlink r:id="rIdSial117" ref="N117"/>
     <x:hyperlink r:id="rIdSial118" ref="N118"/>
   </x:hyperlinks>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
     <x:tablePart r:id="Rf05761c7b56f49be"/>
   </x:tableParts>
@@ -6943,7 +6943,6 @@
       <x:formula>OR(LEFT(G9,3)="غير",LEFT(G9,2)="لم")</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:hyperlinks>
     <x:hyperlink r:id="rIdSial9" ref="N9"/>
     <x:hyperlink r:id="rIdSial10" ref="N10"/>
@@ -6959,6 +6958,7 @@
     <x:hyperlink r:id="rIdSial20" ref="N20"/>
     <x:hyperlink r:id="rIdSial21" ref="N21"/>
   </x:hyperlinks>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
     <x:tablePart r:id="R150eca9fc2b24b80"/>
   </x:tableParts>

</xml_diff>